<commit_message>
Day 2 Part 2: Built interactive KPI card with Data Validation, SUMIFS, and COUNTIFS
</commit_message>
<xml_diff>
--- a/Day2_Sales_Data.xlsx
+++ b/Day2_Sales_Data.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\test_practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{215C4824-334D-4E68-B5B3-E21BC6C1266F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4239DB68-AAFE-4BD9-A73F-052FCD54A7C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6888" yWindow="0" windowWidth="16248" windowHeight="12336" xr2:uid="{3E787063-B8E9-4D18-B9E0-92328B8EC21A}"/>
   </bookViews>
   <sheets>
     <sheet name="Day2_Sales_Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
   <si>
     <t>Order_ID</t>
   </si>
@@ -107,12 +120,24 @@
   </si>
   <si>
     <t>Deal_Type</t>
+  </si>
+  <si>
+    <t>Number of Deals:</t>
+  </si>
+  <si>
+    <t>Select Region:</t>
+  </si>
+  <si>
+    <t>Total Revenue:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;₹&quot;\ #,##0.00;[Red]&quot;₹&quot;\ \-#,##0.00"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -249,7 +274,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -429,8 +454,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -545,6 +576,68 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -590,9 +683,16 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1018,7 +1118,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27EC6945-C2A1-4D0E-927C-DA46BA29D2F2}">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.21875" customWidth="1"/>
@@ -1030,9 +1130,13 @@
     <col min="8" max="8" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.6640625" customWidth="1"/>
+    <col min="16" max="16" width="15" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1069,8 +1173,14 @@
       <c r="N1" t="s">
         <v>25</v>
       </c>
+      <c r="P1" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" s="8" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1001</v>
       </c>
@@ -1111,8 +1221,10 @@
       <c r="N2" s="1">
         <v>0.08</v>
       </c>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="3"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1002</v>
       </c>
@@ -1153,8 +1265,15 @@
       <c r="N3" s="1">
         <v>0.05</v>
       </c>
+      <c r="P3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q3" s="4">
+        <f>SUMIFS(Table1[Total_Revenue],Table1[Region],Q1)</f>
+        <v>250000</v>
+      </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1003</v>
       </c>
@@ -1195,8 +1314,15 @@
       <c r="N4" s="1">
         <v>0.06</v>
       </c>
+      <c r="P4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q4" s="6">
+        <f>COUNTIFS(Table1[Region],Q1)</f>
+        <v>2</v>
+      </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1004</v>
       </c>
@@ -1238,7 +1364,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1005</v>
       </c>
@@ -1280,7 +1406,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1006</v>
       </c>
@@ -1316,7 +1442,7 @@
         <v>High Value</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1007</v>
       </c>
@@ -1352,7 +1478,7 @@
         <v>High Value</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1008</v>
       </c>
@@ -1394,6 +1520,11 @@
       <formula>NOT(ISERROR(SEARCH("High Value",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q1" xr:uid="{581C2F7A-B1C5-43B8-A2B9-17DBF41A2878}">
+      <formula1>"North, South, East, West"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>